<commit_message>
tuned waste functions to scenarios
</commit_message>
<xml_diff>
--- a/output/global_calorie_inadequacy_3scenarios.xlsx
+++ b/output/global_calorie_inadequacy_3scenarios.xlsx
@@ -378,10 +378,10 @@
         </is>
       </c>
       <c r="B2">
-        <v>0.05599416962773597</v>
+        <v>0.06051850666996739</v>
       </c>
       <c r="C2">
-        <v>5.599416962773597</v>
+        <v>6.051850666996739</v>
       </c>
     </row>
     <row r="3">
@@ -391,10 +391,10 @@
         </is>
       </c>
       <c r="B3">
-        <v>0.2309559355042556</v>
+        <v>0.1999251239701637</v>
       </c>
       <c r="C3">
-        <v>23.09559355042556</v>
+        <v>19.99251239701637</v>
       </c>
     </row>
     <row r="4">
@@ -404,10 +404,10 @@
         </is>
       </c>
       <c r="B4">
-        <v>0.08892911814377502</v>
+        <v>0.1017995920748739</v>
       </c>
       <c r="C4">
-        <v>8.892911814377502</v>
+        <v>10.17995920748739</v>
       </c>
     </row>
   </sheetData>

</xml_diff>